<commit_message>
Mise à jour données 2024
</commit_message>
<xml_diff>
--- a/Palmares.xlsx
+++ b/Palmares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Desktop\Trophée DMA\Site vF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E08FF9-2111-4AD6-8163-347680FA536E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBA66DC-E614-48FF-8372-28FD113B580C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="216" yWindow="0" windowWidth="10956" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="101">
   <si>
     <t>ville</t>
   </si>
@@ -202,6 +202,132 @@
   </si>
   <si>
     <t>Finales Nationales Ensisheim</t>
+  </si>
+  <si>
+    <t>Finales Nationales Limoges</t>
+  </si>
+  <si>
+    <t>CYPRIEN PELLIER-CUIT</t>
+  </si>
+  <si>
+    <t>MARTIN PIQUEREZ</t>
+  </si>
+  <si>
+    <t>AMBRE LE MOEL</t>
+  </si>
+  <si>
+    <t>LUCAS GASCARD</t>
+  </si>
+  <si>
+    <t>AUGUSTIN BACH</t>
+  </si>
+  <si>
+    <t>CARLOS TERRONES VEGA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STEPHAN JANY </t>
+  </si>
+  <si>
+    <t>Niveau 10</t>
+  </si>
+  <si>
+    <t>Niveau 12</t>
+  </si>
+  <si>
+    <t>NATHAN HEN</t>
+  </si>
+  <si>
+    <t>CHARLIE MULETA</t>
+  </si>
+  <si>
+    <t>THIMOTHEE NGUYEN</t>
+  </si>
+  <si>
+    <t>GREGOIRE BLANC</t>
+  </si>
+  <si>
+    <t>HUGO MONCHICOURT</t>
+  </si>
+  <si>
+    <t>SYLVESTRE COULEE-ECOCHARD</t>
+  </si>
+  <si>
+    <t>EMMA DUPUIS</t>
+  </si>
+  <si>
+    <t>LEO MARIN</t>
+  </si>
+  <si>
+    <t>OSCAR DUPLAIX</t>
+  </si>
+  <si>
+    <t>ROMANE LABAT</t>
+  </si>
+  <si>
+    <t>ELI LEBARREAU</t>
+  </si>
+  <si>
+    <t>LIAM JOFFRES</t>
+  </si>
+  <si>
+    <t>PAUL FINDEISEN</t>
+  </si>
+  <si>
+    <t>ANDREA FASSINO VACCARO</t>
+  </si>
+  <si>
+    <t>LIONEL BAYARD</t>
+  </si>
+  <si>
+    <t>ELYAS GATET</t>
+  </si>
+  <si>
+    <t>MAIRA ESPOSITO</t>
+  </si>
+  <si>
+    <t>JULIEN ALLARD</t>
+  </si>
+  <si>
+    <t>LENESTOUR NINO</t>
+  </si>
+  <si>
+    <t>FRANCOISE CRESCIONE</t>
+  </si>
+  <si>
+    <t>LEO REY</t>
+  </si>
+  <si>
+    <t>AIDEN STAINER</t>
+  </si>
+  <si>
+    <t>ROMEO BELLON</t>
+  </si>
+  <si>
+    <t>ARMEL BIENACEL</t>
+  </si>
+  <si>
+    <t>ARTHUR MARTINEZ</t>
+  </si>
+  <si>
+    <t>ADRIENCHATEL</t>
+  </si>
+  <si>
+    <t>NILS BIZET</t>
+  </si>
+  <si>
+    <t>LOUIS TROSSAT</t>
+  </si>
+  <si>
+    <t>ANGELO OUDOT</t>
+  </si>
+  <si>
+    <t>Charnècles</t>
+  </si>
+  <si>
+    <t>Niveau 2</t>
+  </si>
+  <si>
+    <t>Niveau 1</t>
   </si>
 </sst>
 </file>
@@ -568,10 +694,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="28.88671875" style="1" customWidth="1"/>
     <col min="4" max="4" width="20.77734375" style="1" customWidth="1"/>
@@ -600,124 +726,84 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="B5" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="B6" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="B8" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -725,16 +811,16 @@
         <v>28</v>
       </c>
       <c r="B9" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>7</v>
@@ -742,79 +828,59 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="B11" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B13" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>8</v>
@@ -822,259 +888,299 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="B14" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="B15" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="B16" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>9</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="B18" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="B19" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="B20" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="B21" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="B23" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="B24" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B26" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="B28" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>8</v>
@@ -1082,156 +1188,176 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="B30" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="B31" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="B32" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" s="1">
-        <v>2025</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="B35" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B36" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>15</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="B38" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B40" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>5</v>
@@ -1242,22 +1368,1042 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B41" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F41" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B48" s="1">
+        <v>2024</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B55" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B56" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B57" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B58" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B62" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B63" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B64" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B65" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B66" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B67" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B68" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B70" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B71" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B72" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B73" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B74" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B75" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B78" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B80" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B81" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B82" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B83" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B84" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B85" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B87" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B88" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B90" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B92" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B93" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B96" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B98" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B100" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B101" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B103" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B104" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B105" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B106" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B108" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B110" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B111" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B113" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B115" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B116" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise à jour des résultats
</commit_message>
<xml_diff>
--- a/Palmares.xlsx
+++ b/Palmares.xlsx
@@ -1,31 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Desktop\Trophée DMA\Site vF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CB6022-5FB7-4A4D-B438-42EB3A8A2298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DCD3B8-8CCA-45BD-9FE6-522DE10F0967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="140">
   <si>
     <t>ville</t>
   </si>
@@ -312,9 +324,6 @@
     <t>LOUIS TROSSAT</t>
   </si>
   <si>
-    <t>ANGELO OUDOT</t>
-  </si>
-  <si>
     <t>Charnècles</t>
   </si>
   <si>
@@ -325,6 +334,129 @@
   </si>
   <si>
     <t>NINO LENESTOUR</t>
+  </si>
+  <si>
+    <t>Magland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAURA PERRET </t>
+  </si>
+  <si>
+    <t xml:space="preserve">YUMA LEMARRE REY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BENJAMIN CHAUDET </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MARCEAU CHOUTEAU </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROBIN KOLODIE </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> THEO GISCLON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELIOT BIBOLLET RUCHE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAEL BRANGER </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> LOLA GISCLON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMBRE LE MOEL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOIC PERRET </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CHARLY BIBOLLET RUCHE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MARCUS DA RIVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> EVA OMNES</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ANGELO OUDOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niveau 8 </t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>GAUVAIN BLANCHARD</t>
+  </si>
+  <si>
+    <t>AIDA CASSEL</t>
+  </si>
+  <si>
+    <t>CAMILLE CITTADINI</t>
+  </si>
+  <si>
+    <t>MATHEO VALLARINO</t>
+  </si>
+  <si>
+    <t>NATHAN BERVOET</t>
+  </si>
+  <si>
+    <t>BAPTISTE ASTIER</t>
+  </si>
+  <si>
+    <t>AUXENCE CALLOT</t>
+  </si>
+  <si>
+    <t>NOEMIE GRANDGUILLOT</t>
+  </si>
+  <si>
+    <t>GHJUVAN CASALTA</t>
+  </si>
+  <si>
+    <t>GASPARD TALLON</t>
+  </si>
+  <si>
+    <t>MAXIME BONNARD</t>
+  </si>
+  <si>
+    <t>DANIEL MAURIN</t>
+  </si>
+  <si>
+    <t>NAIS OBEA MANON</t>
+  </si>
+  <si>
+    <t>RAOUL BARBET</t>
+  </si>
+  <si>
+    <t>ERWANN AILLAUD</t>
+  </si>
+  <si>
+    <t>ELYNA LEDROIT</t>
+  </si>
+  <si>
+    <t>ROMAIN SERRE DUPUY</t>
+  </si>
+  <si>
+    <t>MILAN BLANC</t>
+  </si>
+  <si>
+    <t>ULYSSE VALDIVIA</t>
+  </si>
+  <si>
+    <t>ANTHONY SGUEGLIA</t>
+  </si>
+  <si>
+    <t>IMANOL AUDU</t>
+  </si>
+  <si>
+    <t>RASMUS NOMMENSEN</t>
+  </si>
+  <si>
+    <t>JONAS MURATI</t>
   </si>
 </sst>
 </file>
@@ -426,6 +558,27 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Feuille1"/>
+      <sheetName val="Feuille2"/>
+      <sheetName val="Feuille3"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.6640625" style="1" customWidth="1"/>
@@ -1365,7 +1518,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B41" s="1">
         <v>2024</v>
@@ -2131,10 +2284,10 @@
         <v>2026</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>4</v>
@@ -2151,10 +2304,10 @@
         <v>2026</v>
       </c>
       <c r="C98" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D98" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>5</v>
@@ -2171,7 +2324,7 @@
         <v>2026</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>10</v>
@@ -2191,7 +2344,7 @@
         <v>2026</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>10</v>
@@ -2211,7 +2364,7 @@
         <v>2026</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D103" s="1" t="s">
         <v>12</v>
@@ -2231,7 +2384,7 @@
         <v>2026</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D104" s="1" t="s">
         <v>12</v>
@@ -2251,7 +2404,7 @@
         <v>2026</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>12</v>
@@ -2271,7 +2424,7 @@
         <v>2026</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D106" s="1" t="s">
         <v>12</v>
@@ -2291,7 +2444,7 @@
         <v>2026</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>13</v>
@@ -2311,7 +2464,7 @@
         <v>2026</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D110" s="1" t="s">
         <v>14</v>
@@ -2331,7 +2484,7 @@
         <v>2026</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D111" s="1" t="s">
         <v>14</v>
@@ -2351,7 +2504,7 @@
         <v>2026</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>18</v>
@@ -2371,7 +2524,7 @@
         <v>2026</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D115" s="1" t="s">
         <v>19</v>
@@ -2385,13 +2538,13 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B116" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="B116" s="1">
-        <v>2026</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>19</v>
@@ -2401,6 +2554,806 @@
       </c>
       <c r="F116" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B118" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B120" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B122" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A123" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B123" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B124" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B125" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B126" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A128" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B128" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E128" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A129" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B129" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A130" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B130" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E130" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A132" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B132" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E132" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A133" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B133" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A135" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B135" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A137" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B137" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A139" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B139" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D139" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A141" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B141" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A142" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B142" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D142" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A143" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B143" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D143" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E143" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A144" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B144" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D144" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F144" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A145" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B145" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D145" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A147" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B147" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D147" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E147" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F147" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A148" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B148" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D148" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F148" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A149" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B149" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D149" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A151" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B151" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D151" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F151" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A152" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B152" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D152" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E152" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F152" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A153" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B153" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D153" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A154" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B154" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E154" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F154" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A155" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B155" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D155" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E155" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A157" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B157" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E157" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A158" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B158" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A159" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B159" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A160" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B160" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D160" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E160" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B161" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A163" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B163" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D163" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B164" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D164" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E164" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A166" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B166" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A168" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B168" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D168" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A170" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B170" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A171" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B171" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C171" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D171" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E171" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A173" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B173" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D173" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F173" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>